<commit_message>
Coverage review corrections to matrix v3
Control:     None
Change:      s.8(4) moved to DPDP-Act-S8(1); s.27(2) duty to comply with Board directions added to DPDP-Act-S32; s.33 shown as applying to companies; s.7(b), 7(c) removed from DPDP-Act-S7; Rule 12 citation corrected; Rules 14(1), 14(2) added to DPDP-Act-S12; Consent Managers added to Rule 14 lines; wording corrections to S5(1), S5(2), S9(1), S9(3) and four Coverage notes.
Reason:      Independent review of every Coverage line against the Gazette text.
Tested by:   Recalculated with no formula errors; all legal-text links checked.
Approved by: Rituraj
</commit_message>
<xml_diff>
--- a/blueprint/DPDP_Obligations_Matrix.xlsx
+++ b/blueprint/DPDP_Obligations_Matrix.xlsx
@@ -20,7 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Obligations Matrix'!$A$4:$W$44</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Legal Text'!$A$4:$D$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Legal Text'!$A$4:$D$65</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Event Playbook'!$A$4:$H$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Coverage'!$A$4:$G$89</definedName>
   </definedNames>
@@ -1580,7 +1580,7 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>Act s.7(a) to s.7(i)</t>
+          <t>Act s.7(a), s.7(d) to s.7(i)</t>
         </is>
       </c>
       <c r="F6" s="11" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Every request for consent must come with, or after, a notice that lists the personal data, the purpose, the goods or services it enables, and how to withdraw consent, exercise rights and complain to the Data Protection Board. The notice must stand on its own and be in clear, plain language, in English or a language in the Eighth Schedule to the Constitution.</t>
+          <t>Every request for consent must come with, or after, a notice that lists the personal data, the purpose, the goods or services it enables, and how to withdraw consent, exercise rights and complain to the Data Protection Board. The request for consent must give the contact details of the Data Protection Officer, where applicable, or of another person authorised to respond (s.6(3)). The notice and the request must be in clear, plain language, with the option to read them in English or any language in the Eighth Schedule to the Constitution.</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
@@ -1781,7 +1781,7 @@
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
-          <t>DPDP-Act-S5(1)</t>
+          <t>DPDP-Act-S5(1) (Rule 3 sets the content of every notice, including this one)</t>
         </is>
       </c>
       <c r="G8" s="12">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>The Data Fiduciary remains responsible for compliance even for processing done on its behalf by Data Processors. It may use a Data Processor only under a valid contract.</t>
+          <t>The Data Fiduciary remains responsible for compliance even for processing done on its behalf by Data Processors. It may use a Data Processor only under a valid contract. It must also put in place technical and organisational measures to make sure the Act and the Rules are observed in practice (s.8(4)).</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
@@ -2266,12 +2266,12 @@
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>Act s.8(1), s.8(2)</t>
+          <t>Act s.8(1), s.8(2), s.8(4)</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>DPDP-Rule-6(1)(f) (security terms in processor contracts)</t>
+          <t>DPDP-Rule-6(1)(f) (security terms in processor contracts); DPDP-Act-S8(5)</t>
         </is>
       </c>
       <c r="G13" s="12">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="N13" s="11" t="inlineStr">
         <is>
-          <t>Keep a register of every vendor that receives personal data. Use standard contract clauses covering security, erasure and breach notification.</t>
+          <t>Keep a register of every vendor that receives personal data. Use standard contract clauses covering security, erasure and breach notification. Run a compliance programme for the Act as a whole: a named owner for each duty, periodic review, and records that show it works.</t>
         </is>
       </c>
       <c r="O13" s="11" t="inlineStr">
@@ -2318,7 +2318,7 @@
       </c>
       <c r="P13" s="11" t="inlineStr">
         <is>
-          <t>Signed contracts; vendor register.</t>
+          <t>Signed contracts; vendor register. Compliance programme records and review minutes.</t>
         </is>
       </c>
       <c r="Q13" s="13" t="n">
@@ -2373,7 +2373,7 @@
         </is>
       </c>
       <c r="G14" s="12">
-        <f>HYPERLINK("#'Legal Text'!A16","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A17","Read the exact text")</f>
         <v/>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -2471,7 +2471,7 @@
         </is>
       </c>
       <c r="G15" s="12">
-        <f>HYPERLINK("#'Legal Text'!A17","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A18","Read the exact text")</f>
         <v/>
       </c>
       <c r="H15" s="11" t="inlineStr">
@@ -2569,7 +2569,7 @@
         </is>
       </c>
       <c r="G16" s="12">
-        <f>HYPERLINK("#'Legal Text'!A18","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A19","Read the exact text")</f>
         <v/>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -2648,7 +2648,7 @@
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Protect personal data with reasonable security safeguards to prevent a breach. At a minimum: encryption, masking or tokenisation; access control; logs, monitoring and review; backups for continuity; keeping logs and personal data for one year for detection and investigation; security clauses in Data Processor contracts; and technical and organisational measures.</t>
+          <t>Protect personal data with reasonable security safeguards to prevent a breach. At a minimum: encryption, masking or tokenisation; access control; logs, monitoring and review; backups for continuity; keeping logs and personal data for one year for detection and investigation; security clauses in Data Processor contracts; and measures to make sure the safeguards are observed.</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
@@ -2658,7 +2658,7 @@
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>Act s.8(4), s.8(5); Rules 6(2). Each clause of Rule 6(1) has its own row.</t>
+          <t>Act s.8(5); Rules 6(2). Each clause of Rule 6(1) has its own row.</t>
         </is>
       </c>
       <c r="F17" s="11" t="inlineStr">
@@ -2667,7 +2667,7 @@
         </is>
       </c>
       <c r="G17" s="12">
-        <f>HYPERLINK("#'Legal Text'!A19","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A20","Read the exact text")</f>
         <v/>
       </c>
       <c r="H17" s="11" t="inlineStr">
@@ -2765,7 +2765,7 @@
         </is>
       </c>
       <c r="G18" s="12">
-        <f>HYPERLINK("#'Legal Text'!A20","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A21","Read the exact text")</f>
         <v/>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -2863,7 +2863,7 @@
         </is>
       </c>
       <c r="G19" s="12">
-        <f>HYPERLINK("#'Legal Text'!A21","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A22","Read the exact text")</f>
         <v/>
       </c>
       <c r="H19" s="11" t="inlineStr">
@@ -2961,7 +2961,7 @@
         </is>
       </c>
       <c r="G20" s="12">
-        <f>HYPERLINK("#'Legal Text'!A22","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A23","Read the exact text")</f>
         <v/>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -3059,7 +3059,7 @@
         </is>
       </c>
       <c r="G21" s="12">
-        <f>HYPERLINK("#'Legal Text'!A23","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A24","Read the exact text")</f>
         <v/>
       </c>
       <c r="H21" s="11" t="inlineStr">
@@ -3157,7 +3157,7 @@
         </is>
       </c>
       <c r="G22" s="12">
-        <f>HYPERLINK("#'Legal Text'!A24","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A25","Read the exact text")</f>
         <v/>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -3265,7 +3265,7 @@
         </is>
       </c>
       <c r="G23" s="12">
-        <f>HYPERLINK("#'Legal Text'!A25","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A26","Read the exact text")</f>
         <v/>
       </c>
       <c r="H23" s="11" t="inlineStr">
@@ -3363,7 +3363,7 @@
         </is>
       </c>
       <c r="G24" s="12">
-        <f>HYPERLINK("#'Legal Text'!A26","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A27","Read the exact text")</f>
         <v/>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -3461,7 +3461,7 @@
         </is>
       </c>
       <c r="G25" s="12">
-        <f>HYPERLINK("#'Legal Text'!A27","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A28","Read the exact text")</f>
         <v/>
       </c>
       <c r="H25" s="11" t="inlineStr">
@@ -3559,7 +3559,7 @@
         </is>
       </c>
       <c r="G26" s="12">
-        <f>HYPERLINK("#'Legal Text'!A29","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A30","Read the exact text")</f>
         <v/>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -3657,7 +3657,7 @@
         </is>
       </c>
       <c r="G27" s="12">
-        <f>HYPERLINK("#'Legal Text'!A30","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A31","Read the exact text")</f>
         <v/>
       </c>
       <c r="H27" s="11" t="inlineStr">
@@ -3755,7 +3755,7 @@
         </is>
       </c>
       <c r="G28" s="12">
-        <f>HYPERLINK("#'Legal Text'!A31","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A32","Read the exact text")</f>
         <v/>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -3853,7 +3853,7 @@
         </is>
       </c>
       <c r="G29" s="12">
-        <f>HYPERLINK("#'Legal Text'!A32","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A33","Read the exact text")</f>
         <v/>
       </c>
       <c r="H29" s="11" t="inlineStr">
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="G30" s="12">
-        <f>HYPERLINK("#'Legal Text'!A35","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A36","Read the exact text")</f>
         <v/>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -4049,7 +4049,7 @@
         </is>
       </c>
       <c r="G31" s="12">
-        <f>HYPERLINK("#'Legal Text'!A37","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A38","Read the exact text")</f>
         <v/>
       </c>
       <c r="H31" s="11" t="inlineStr">
@@ -4138,7 +4138,7 @@
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>Act s.12(1), s.12(2)(a) to (c), s.12(3)</t>
+          <t>Act s.12(1), s.12(2)(a) to (c), s.12(3); Rules 14(1), 14(2)</t>
         </is>
       </c>
       <c r="F32" s="11" t="inlineStr">
@@ -4147,7 +4147,7 @@
         </is>
       </c>
       <c r="G32" s="12">
-        <f>HYPERLINK("#'Legal Text'!A40","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A41","Read the exact text")</f>
         <v/>
       </c>
       <c r="H32" s="11" t="inlineStr">
@@ -4245,7 +4245,7 @@
         </is>
       </c>
       <c r="G33" s="12">
-        <f>HYPERLINK("#'Legal Text'!A42","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A43","Read the exact text")</f>
         <v/>
       </c>
       <c r="H33" s="11" t="inlineStr">
@@ -4343,7 +4343,7 @@
         </is>
       </c>
       <c r="G34" s="12">
-        <f>HYPERLINK("#'Legal Text'!A45","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A46","Read the exact text")</f>
         <v/>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>Before processing any personal data of a child (under 18), obtain the verifiable consent of a parent, after checking that the parent is an identifiable adult, using the Data Fiduciary's own reliable records or identity and age details or a token from an authorised entity such as DigiLocker.</t>
+          <t>Before processing any personal data of a child (under 18), obtain the verifiable consent of a parent (or, for a person with disability, of her lawful guardian: see DPDP-Rule-11(1)), after checking that the parent is an identifiable adult, using the Data Fiduciary's own reliable records or identity and age details or a token from an authorised entity such as DigiLocker.</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr">
@@ -4437,11 +4437,11 @@
       </c>
       <c r="F35" s="11" t="inlineStr">
         <is>
-          <t>DPDP-Rule-11(1); DPDP-Act-S9(3)</t>
+          <t>DPDP-Rule-11(1); DPDP-Act-S9(3) (the Fourth Schedule exemptions under Rule 12 also lift s.9(1))</t>
         </is>
       </c>
       <c r="G35" s="12">
-        <f>HYPERLINK("#'Legal Text'!A46","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A47","Read the exact text")</f>
         <v/>
       </c>
       <c r="H35" s="11" t="inlineStr">
@@ -4451,7 +4451,7 @@
       </c>
       <c r="I35" s="11" t="inlineStr">
         <is>
-          <t>Data Fiduciaries that process children's personal data</t>
+          <t>Data Fiduciaries that process personal data of children, or of persons with disability who have a lawful guardian</t>
         </is>
       </c>
       <c r="J35" s="11" t="inlineStr">
@@ -4520,7 +4520,7 @@
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Do not process a child's data in a way likely to harm her well-being. Do not track, behaviourally monitor, or target advertising at children, unless an exemption in the Fourth Schedule applies (for example healthcare, education or safety).</t>
+          <t>Do not process a child's data in a way likely to harm her well-being; no exemption lifts this duty. Do not track, behaviourally monitor, or target advertising at children, unless an exemption in the Fourth Schedule applies (for example healthcare, education or safety).</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -4530,7 +4530,7 @@
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>Act s.9(2), s.9(3), s.9(4), s.9(5); Rules 12(1) to 12(3); Fourth Schedule, Parts A and B</t>
+          <t>Act s.9(2), s.9(3), s.9(4), s.9(5); Rules 12(1), 12(2); Fourth Schedule, Parts A and B</t>
         </is>
       </c>
       <c r="F36" s="11" t="inlineStr">
@@ -4539,7 +4539,7 @@
         </is>
       </c>
       <c r="G36" s="12">
-        <f>HYPERLINK("#'Legal Text'!A48","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A49","Read the exact text")</f>
         <v/>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="G37" s="12">
-        <f>HYPERLINK("#'Legal Text'!A50","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A51","Read the exact text")</f>
         <v/>
       </c>
       <c r="H37" s="11" t="inlineStr">
@@ -4735,7 +4735,7 @@
         </is>
       </c>
       <c r="G38" s="12">
-        <f>HYPERLINK("#'Legal Text'!A51","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A52","Read the exact text")</f>
         <v/>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -4833,7 +4833,7 @@
         </is>
       </c>
       <c r="G39" s="12">
-        <f>HYPERLINK("#'Legal Text'!A52","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A53","Read the exact text")</f>
         <v/>
       </c>
       <c r="H39" s="11" t="inlineStr">
@@ -4931,7 +4931,7 @@
         </is>
       </c>
       <c r="G40" s="12">
-        <f>HYPERLINK("#'Legal Text'!A53","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A54","Read the exact text")</f>
         <v/>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -5029,7 +5029,7 @@
         </is>
       </c>
       <c r="G41" s="12">
-        <f>HYPERLINK("#'Legal Text'!A55","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A56","Read the exact text")</f>
         <v/>
       </c>
       <c r="H41" s="11" t="inlineStr">
@@ -5108,7 +5108,7 @@
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>The Data Protection Board can inquire, give directions and accept a voluntary undertaking, which bars proceedings on its contents; breaking the undertaking is itself a breach. Appeals against Board orders go to the Appellate Tribunal within 60 days.</t>
+          <t>A company must comply with any direction the Data Protection Board issues to it, including urgent remedial measures after a breach (s.27(1)(a), s.27(2)). The Data Protection Board can inquire, give directions and accept a voluntary undertaking, which bars proceedings on its contents; breaking the undertaking is itself a breach. Appeals against Board orders go to the Appellate Tribunal within 60 days.</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -5127,7 +5127,7 @@
         </is>
       </c>
       <c r="G42" s="12">
-        <f>HYPERLINK("#'Legal Text'!A57","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A58","Read the exact text")</f>
         <v/>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -5160,7 +5160,7 @@
       </c>
       <c r="N42" s="11" t="inlineStr">
         <is>
-          <t>Procedure for dealing with the Board; legal adviser identified in advance.</t>
+          <t>Procedure for dealing with the Board; legal adviser identified in advance. Keep a log of every Board direction and the action taken.</t>
         </is>
       </c>
       <c r="O42" s="11" t="inlineStr">
@@ -5170,7 +5170,7 @@
       </c>
       <c r="P42" s="11" t="inlineStr">
         <is>
-          <t>Correspondence file.</t>
+          <t>Correspondence file. Log of Board directions and evidence of compliance.</t>
         </is>
       </c>
       <c r="Q42" s="13" t="n">
@@ -5225,7 +5225,7 @@
         </is>
       </c>
       <c r="G43" s="12">
-        <f>HYPERLINK("#'Legal Text'!A60","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A62","Read the exact text")</f>
         <v/>
       </c>
       <c r="H43" s="11" t="inlineStr">
@@ -5323,7 +5323,7 @@
         </is>
       </c>
       <c r="G44" s="12">
-        <f>HYPERLINK("#'Legal Text'!A62","Read the exact text")</f>
+        <f>HYPERLINK("#'Legal Text'!A64","Read the exact text")</f>
         <v/>
       </c>
       <c r="H44" s="11" t="inlineStr">
@@ -5438,7 +5438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5728,39 +5728,39 @@
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
+          <t>DPDP-Act-S8(1)</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Digital Personal Data Protection Act, 2023, Section 8(4)</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>(4) A Data Fiduciary shall implement appropriate technical and organisational measures to ensure effective observance of the provisions of this Act and the rules made thereunder.</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
           <t>DPDP-Act-S8(3)</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Act, 2023, Section 8(3)</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>(3) Where personal data processed by a Data Fiduciary is likely to be— (a) used to make a decision that affects the Data Principal; or (b) disclosed to another Data Fiduciary, the Data Fiduciary processing such personal data shall ensure its completeness, accuracy and consistency.</t>
-        </is>
-      </c>
-      <c r="D16" s="11" t="inlineStr">
-        <is>
-          <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="56" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>DPDP-Act-S38</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>Digital Personal Data Protection Act, 2023, Section 38</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
-          <t>38. (1) The provisions of this Act shall be in addition to and not in derogation of any other law for the time being in force. (2) In the event of any conflict between a provision of this Act and a provision of any other law for the time being in force, the provision of this Act shall prevail to the extent of such conflict.</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
@@ -5772,105 +5772,105 @@
     <row r="18" ht="56" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
+          <t>DPDP-Act-S38</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Digital Personal Data Protection Act, 2023, Section 38</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>38. (1) The provisions of this Act shall be in addition to and not in derogation of any other law for the time being in force. (2) In the event of any conflict between a provision of this Act and a provision of any other law for the time being in force, the provision of this Act shall prevail to the extent of such conflict.</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="56" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
           <t>DPDP-Act-S44(2)</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Act, 2023, Section 44(2)</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>(2) The Information Technology Act, 2000 shall be amended in the following manner, namely:— (a) section 43A shall be omitted; (b) in section 81, in the proviso, after the words and figures "the Patents Act, 1970", the words and figures "or the Digital Personal Data Protection Act, 2023" shall be inserted; and (c) in section 87, in sub-section (2), clause (ob) shall be omitted.</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="D19" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="70" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S8(5)</t>
         </is>
       </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>Digital Personal Data Protection Act, 2023, Section 8(4) and Section 8(5)</t>
-        </is>
-      </c>
-      <c r="C19" s="11" t="inlineStr">
-        <is>
-          <t>(4) A Data Fiduciary shall implement appropriate technical and organisational measures to ensure effective observance of the provisions of this Act and the rules made thereunder. (5) A Data Fiduciary shall protect personal data in its possession or under its control, including in respect of any processing undertaken by it or on its behalf by a Data Processor, by taking reasonable security safeguards to prevent personal data breach.</t>
-        </is>
-      </c>
-      <c r="D19" s="11" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Digital Personal Data Protection Act, 2023, Section 8(5)</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>(5) A Data Fiduciary shall protect personal data in its possession or under its control, including in respect of any processing undertaken by it or on its behalf by a Data Processor, by taking reasonable security safeguards to prevent personal data breach.</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="70" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>DPDP-Rule-6(1)(a)</t>
-        </is>
-      </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>Digital Personal Data Protection Rules, 2025, Rule 6(1)(a)</t>
-        </is>
-      </c>
-      <c r="C20" s="11" t="inlineStr">
-        <is>
-          <t>(1) A Data Fiduciary shall protect personal data in its possession or under its control, including in respect of any processing undertaken by it or on its behalf by a Data Processor, by taking reasonable security safeguards to prevent personal data breach, which shall include, at the minimum, — … (a) appropriate data security measures, such as securing of personal data through encryption, obfuscation, masking or the use of virtual tokens mapped to that personal data;</t>
-        </is>
-      </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
         </is>
       </c>
     </row>
     <row r="21" ht="70" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
+          <t>DPDP-Rule-6(1)(a)</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Digital Personal Data Protection Rules, 2025, Rule 6(1)(a)</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>(1) A Data Fiduciary shall protect personal data in its possession or under its control, including in respect of any processing undertaken by it or on its behalf by a Data Processor, by taking reasonable security safeguards to prevent personal data breach, which shall include, at the minimum, — … (a) appropriate data security measures, such as securing of personal data through encryption, obfuscation, masking or the use of virtual tokens mapped to that personal data;</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="70" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
           <t>DPDP-Rule-6(1)(b)</t>
         </is>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Rules, 2025, Rule 6(1)(b)</t>
         </is>
       </c>
-      <c r="C21" s="11" t="inlineStr">
+      <c r="C22" s="11" t="inlineStr">
         <is>
           <t>(1) A Data Fiduciary shall protect personal data in its possession or under its control, including in respect of any processing undertaken by it or on its behalf by a Data Processor, by taking reasonable security safeguards to prevent personal data breach, which shall include, at the minimum, — … (b) appropriate measures to control access to the computer resources used by such Data Fiduciary or such a Data Processor, wherever applicable;</t>
-        </is>
-      </c>
-      <c r="D21" s="11" t="inlineStr">
-        <is>
-          <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="84" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>DPDP-Rule-6(1)(c)</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>Digital Personal Data Protection Rules, 2025, Rule 6(1)(c)</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="inlineStr">
-        <is>
-          <t>(1) A Data Fiduciary shall protect personal data in its possession or under its control, including in respect of any processing undertaken by it or on its behalf by a Data Processor, by taking reasonable security safeguards to prevent personal data breach, which shall include, at the minimum, — … (c) visibility on the accessing of such personal data, through appropriate logs, monitoring and review, for enabling detection of unauthorised access, its investigation and remediation to prevent recurrence;</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -5882,907 +5882,951 @@
     <row r="23" ht="84" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
+          <t>DPDP-Rule-6(1)(c)</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Digital Personal Data Protection Rules, 2025, Rule 6(1)(c)</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>(1) A Data Fiduciary shall protect personal data in its possession or under its control, including in respect of any processing undertaken by it or on its behalf by a Data Processor, by taking reasonable security safeguards to prevent personal data breach, which shall include, at the minimum, — … (c) visibility on the accessing of such personal data, through appropriate logs, monitoring and review, for enabling detection of unauthorised access, its investigation and remediation to prevent recurrence;</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="84" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
           <t>DPDP-Rule-6(1)(d)</t>
         </is>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Rules, 2025, Rule 6(1)(d)</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr">
+      <c r="C24" s="11" t="inlineStr">
         <is>
           <t>(1) A Data Fiduciary shall protect personal data in its possession or under its control, including in respect of any processing undertaken by it or on its behalf by a Data Processor, by taking reasonable security safeguards to prevent personal data breach, which shall include, at the minimum, — … (d) reasonable measures for continued processing in the event of confidentiality, integrity or availability of such personal data being compromised as a result of destruction or loss of access to personal data or otherwise, such as by way of data-backups;</t>
         </is>
       </c>
-      <c r="D23" s="11" t="inlineStr">
+      <c r="D24" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="98" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
+    <row r="25" ht="98" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>DPDP-Rule-6(1)(e)</t>
         </is>
       </c>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Rules, 2025, Rule 6(1)(e)</t>
         </is>
       </c>
-      <c r="C24" s="11" t="inlineStr">
+      <c r="C25" s="11" t="inlineStr">
         <is>
           <t>(1) A Data Fiduciary shall protect personal data in its possession or under its control, including in respect of any processing undertaken by it or on its behalf by a Data Processor, by taking reasonable security safeguards to prevent personal data breach, which shall include, at the minimum, — … (e) for enabling the detection of unauthorised access, its investigation, remediation to prevent recurrence and continued processing in the event of such a compromise, retain such logs and personal data for a period of one year, unless compliance with any law for the time being in force requires otherwise;</t>
         </is>
       </c>
-      <c r="D24" s="11" t="inlineStr">
+      <c r="D25" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="84" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
+    <row r="26" ht="84" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>DPDP-Rule-6(1)(f)</t>
         </is>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Rules, 2025, Rule 6(1)(f)</t>
         </is>
       </c>
-      <c r="C25" s="11" t="inlineStr">
+      <c r="C26" s="11" t="inlineStr">
         <is>
           <t>(1) A Data Fiduciary shall protect personal data in its possession or under its control, including in respect of any processing undertaken by it or on its behalf by a Data Processor, by taking reasonable security safeguards to prevent personal data breach, which shall include, at the minimum, — … (f) appropriate provision in the contract entered into between such Data Fiduciary and such a Data Processor, wherever applicable, for taking reasonable security safeguards; and</t>
         </is>
       </c>
-      <c r="D25" s="11" t="inlineStr">
+      <c r="D26" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="70" customHeight="1">
-      <c r="A26" s="5" t="inlineStr">
+    <row r="27" ht="70" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>DPDP-Rule-6(1)(g)</t>
         </is>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Rules, 2025, Rule 6(1)(g)</t>
         </is>
       </c>
-      <c r="C26" s="11" t="inlineStr">
+      <c r="C27" s="11" t="inlineStr">
         <is>
           <t>(1) A Data Fiduciary shall protect personal data in its possession or under its control, including in respect of any processing undertaken by it or on its behalf by a Data Processor, by taking reasonable security safeguards to prevent personal data breach, which shall include, at the minimum, — … (g) appropriate technical and organisational measures to ensure effective observance of security safeguards.</t>
         </is>
       </c>
-      <c r="D26" s="11" t="inlineStr">
+      <c r="D27" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="45" customHeight="1">
-      <c r="A27" s="5" t="inlineStr">
+    <row r="28" ht="45" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>DPDP-Rule-7(1)</t>
         </is>
       </c>
-      <c r="B27" s="11" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Act, 2023, Section 8(6)</t>
         </is>
       </c>
-      <c r="C27" s="11" t="inlineStr">
+      <c r="C28" s="11" t="inlineStr">
         <is>
           <t>(6) In the event of a personal data breach, the Data Fiduciary shall give the Board and each affected Data Principal, intimation of such breach in such form and manner as may be prescribed.</t>
         </is>
       </c>
-      <c r="D27" s="11" t="inlineStr">
+      <c r="D28" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="126" customHeight="1">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>DPDP-Rule-7(1)</t>
-        </is>
-      </c>
-      <c r="B28" s="11" t="inlineStr">
-        <is>
-          <t>Digital Personal Data Protection Rules, 2025, Rule 7(1)</t>
-        </is>
-      </c>
-      <c r="C28" s="11" t="inlineStr">
-        <is>
-          <t>(1) On becoming aware of any personal data breach, the Data Fiduciary shall, to the best of its knowledge, intimate to each affected Data Principal, in a concise, clear and plain manner and without delay, through her user account or any mode of communication registered by her with the Data Fiduciary, — (a) a description of the breach, including its nature, extent and the timing of its occurrence; (b) the consequences relevant to her, that are likely to arise from the breach; (c) the measures implemented and being implemented by the Data Fiduciary, if any, to mitigate risk; (d) the safety measures that she may take to protect her interests; and (e) business contact information of a person who is able to respond on behalf of the Data Fiduciary, to queries, if any, of the Data Principal.</t>
-        </is>
-      </c>
-      <c r="D28" s="11" t="inlineStr">
-        <is>
-          <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
         </is>
       </c>
     </row>
     <row r="29" ht="126" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
+          <t>DPDP-Rule-7(1)</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Digital Personal Data Protection Rules, 2025, Rule 7(1)</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>(1) On becoming aware of any personal data breach, the Data Fiduciary shall, to the best of its knowledge, intimate to each affected Data Principal, in a concise, clear and plain manner and without delay, through her user account or any mode of communication registered by her with the Data Fiduciary, — (a) a description of the breach, including its nature, extent and the timing of its occurrence; (b) the consequences relevant to her, that are likely to arise from the breach; (c) the measures implemented and being implemented by the Data Fiduciary, if any, to mitigate risk; (d) the safety measures that she may take to protect her interests; and (e) business contact information of a person who is able to respond on behalf of the Data Fiduciary, to queries, if any, of the Data Principal.</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="126" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
           <t>DPDP-Rule-7(2)</t>
         </is>
       </c>
-      <c r="B29" s="11" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Rules, 2025, Rule 7(2)</t>
         </is>
       </c>
-      <c r="C29" s="11" t="inlineStr">
+      <c r="C30" s="11" t="inlineStr">
         <is>
           <t>(2) On becoming aware of any personal data breach, the Data Fiduciary shall intimate to the Board, — (a) without delay, a description of the breach, including its nature, extent, timing and location of occurrence and the likely impact; (b) within seventy-two hours of becoming aware of the breach, or within such longer period as the Board may allow on a request made in writing in this behalf, — (i) updated and detailed information in respect of such description; (ii) the broad facts related to the events, circumstances and reasons leading to the breach; (iii) measures implemented or proposed, if any, to mitigate risk; (iv) any findings regarding the person who caused the breach; (v) remedial measures taken to prevent recurrence of such breach; and (vi) a report regarding the intimations given to affected Data Principals.</t>
         </is>
       </c>
-      <c r="D29" s="11" t="inlineStr">
+      <c r="D30" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="70" customHeight="1">
-      <c r="A30" s="5" t="inlineStr">
+    <row r="31" ht="70" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S8(7)</t>
         </is>
       </c>
-      <c r="B30" s="11" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Act, 2023, Section 8(7)</t>
         </is>
       </c>
-      <c r="C30" s="11" t="inlineStr">
+      <c r="C31" s="11" t="inlineStr">
         <is>
           <t>(7) A Data Fiduciary shall, unless retention is necessary for compliance with any law for the time being in force,— (a) erase personal data, upon the Data Principal withdrawing her consent or as soon as it is reasonable to assume that the specified purpose is no longer being served, whichever is earlier; and (b) cause its Data Processor to erase any personal data that was made available by the Data Fiduciary for processing to such Data Processor.</t>
         </is>
       </c>
-      <c r="D30" s="11" t="inlineStr">
+      <c r="D31" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="196" customHeight="1">
-      <c r="A31" s="5" t="inlineStr">
+    <row r="32" ht="196" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>DPDP-Rule-8(3)</t>
         </is>
       </c>
-      <c r="B31" s="11" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Rules, 2025, Rule 8(3), with its Illustration</t>
         </is>
       </c>
-      <c r="C31" s="11" t="inlineStr">
+      <c r="C32" s="11" t="inlineStr">
         <is>
           <t>(3) Without prejudice to sub-rules (1) and (2), a Data Fiduciary shall retain, in respect of any processing of personal data undertaken by it or on its behalf by a Data Processor, such personal data, associated traffic data and other logs of the processing for a minimum period of one year from the date of such processing, for the purposes as specified in the Seventh Schedule, after which the Data Fiduciary shall cause such personal data and logs to be erased, unless further retention is required for compliance with any other law for the time being in force or notified by the Government. Illustration. Case 1: X, a Data Principal purchases an e-book on an e-book platform Y. Once delivery is completed, the specified purpose of processing is served. The platform Y must retain the order details, personal data, and logs of the processing (such as order confirmation, payment, and delivery events) for at least one year from the date of the transaction, even if X deletes her account. Case 2: X, a company engages a cloud service provider C as its Data Processor to host customer records. X as the Data Fiduciary, is required to ensure that the C also retains the data and associated logs for at least one year before erasure, unless any other applicable law requires a longer period.</t>
         </is>
       </c>
-      <c r="D31" s="11" t="inlineStr">
+      <c r="D32" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="70" customHeight="1">
-      <c r="A32" s="5" t="inlineStr">
+    <row r="33" ht="70" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>DPDP-Rule-8(1)</t>
         </is>
       </c>
-      <c r="B32" s="11" t="inlineStr">
+      <c r="B33" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Act, 2023, Section 8(8)</t>
         </is>
       </c>
-      <c r="C32" s="11" t="inlineStr">
+      <c r="C33" s="11" t="inlineStr">
         <is>
           <t>(8) The purpose referred to in clause (a) of sub-section (7) shall be deemed to no longer be served, if the Data Principal does not— (a) approach the Data Fiduciary for the performance of the specified purpose; and (b) exercise any of her rights in relation to such processing, for such time period as may be prescribed, and different time periods may be prescribed for different classes of Data Fiduciaries and for different purposes.</t>
         </is>
       </c>
-      <c r="D32" s="11" t="inlineStr">
+      <c r="D33" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="154" customHeight="1">
-      <c r="A33" s="5" t="inlineStr">
+    <row r="34" ht="154" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>DPDP-Rule-8(1)</t>
         </is>
       </c>
-      <c r="B33" s="11" t="inlineStr">
+      <c r="B34" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Rules, 2025, Rule 8(1) and 8(2)</t>
         </is>
       </c>
-      <c r="C33" s="11" t="inlineStr">
+      <c r="C34" s="11" t="inlineStr">
         <is>
           <t>(1) A Data Fiduciary, who is of such class and is processing personal data for such corresponding purposes as are specified in Third Schedule, shall erase such personal data, unless its retention is necessary for compliance with any law for the time being in force, or, for the corresponding time period specified in the Third Schedule, if the Data Principal neither approaches such Data Fiduciary for the performance of the specified purpose nor exercises her rights in relation to such processing. (2) At least forty-eight hours before completion of the time period for erasure of personal data under this rule, the Data Fiduciary shall inform the Data Principal that such personal data shall be erased upon completion of such period, unless she logs into her user account or otherwise initiates contact with the Data Fiduciary for the performance of the specified purpose or exercises her rights in relation to the processing of such personal data.</t>
         </is>
       </c>
-      <c r="D33" s="11" t="inlineStr">
+      <c r="D34" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="56" customHeight="1">
-      <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>DPDP-Rule-8(1)</t>
-        </is>
-      </c>
-      <c r="B34" s="11" t="inlineStr">
-        <is>
-          <t>Digital Personal Data Protection Act, 2023, Section 8(11)</t>
-        </is>
-      </c>
-      <c r="C34" s="11" t="inlineStr">
-        <is>
-          <t>(11) For the purposes of this section, it is hereby clarified that a Data Principal shall be considered as not having approached the Data Fiduciary for the performance of the specified purpose, in any period during which she has not initiated contact with the Data Fiduciary for such performance, in person or by way of communication in electronic or physical form.</t>
-        </is>
-      </c>
-      <c r="D34" s="11" t="inlineStr">
-        <is>
-          <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
         </is>
       </c>
     </row>
     <row r="35" ht="56" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
         <is>
+          <t>DPDP-Rule-8(1)</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>Digital Personal Data Protection Act, 2023, Section 8(11)</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>(11) For the purposes of this section, it is hereby clarified that a Data Principal shall be considered as not having approached the Data Fiduciary for the performance of the specified purpose, in any period during which she has not initiated contact with the Data Fiduciary for such performance, in person or by way of communication in electronic or physical form.</t>
+        </is>
+      </c>
+      <c r="D35" s="11" t="inlineStr">
+        <is>
+          <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="56" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
           <t>DPDP-Rule-9</t>
         </is>
       </c>
-      <c r="B35" s="11" t="inlineStr">
+      <c r="B36" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Act, 2023, Section 8(9)</t>
         </is>
       </c>
-      <c r="C35" s="11" t="inlineStr">
+      <c r="C36" s="11" t="inlineStr">
         <is>
           <t>(9) A Data Fiduciary shall publish, in such manner as may be prescribed, the business contact information of a Data Protection Officer, if applicable, or a person who is able to answer on behalf of the Data Fiduciary, the questions, if any, raised by the Data Principal about the processing of her personal data.</t>
         </is>
       </c>
-      <c r="D35" s="11" t="inlineStr">
+      <c r="D36" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="84" customHeight="1">
-      <c r="A36" s="5" t="inlineStr">
+    <row r="37" ht="84" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>DPDP-Rule-9</t>
         </is>
       </c>
-      <c r="B36" s="11" t="inlineStr">
+      <c r="B37" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Rules, 2025, Rule 9</t>
         </is>
       </c>
-      <c r="C36" s="11" t="inlineStr">
+      <c r="C37" s="11" t="inlineStr">
         <is>
           <t>9. Contact information of person to answer questions about processing.— Every Data Fiduciary shall prominently publish on its website or app, and mention in every response to a communication for the exercise of the rights of a Data Principal under the Act, the business contact information of the Data Protection Officer, if applicable, or a person who is able to answer on behalf of the Data Fiduciary the questions of the Data Principal about the processing of her personal data.</t>
         </is>
       </c>
-      <c r="D36" s="11" t="inlineStr">
+      <c r="D37" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="126" customHeight="1">
-      <c r="A37" s="5" t="inlineStr">
+    <row r="38" ht="126" customHeight="1">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S11(1)</t>
         </is>
       </c>
-      <c r="B37" s="11" t="inlineStr">
+      <c r="B38" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Act, 2023, Section 11(1)</t>
         </is>
       </c>
-      <c r="C37" s="11" t="inlineStr">
+      <c r="C38" s="11" t="inlineStr">
         <is>
           <t>(1) The Data Principal shall have the right to obtain from the Data Fiduciary to whom she has previously given consent, including consent as referred to in clause (a) of section 7 (hereinafter referred to as the said Data Fiduciary), for processing of personal data, upon making to it a request in such manner as may be prescribed,— (a) a summary of personal data which is being processed by such Data Fiduciary and the processing activities undertaken by that Data Fiduciary with respect to such personal data; (b) the identities of all other Data Fiduciaries and Data Processors with whom the personal data has been shared by such Data Fiduciary, along with a description of the personal data so shared; and (c) any other information related to the personal data of such Data Principal and its processing, as may be prescribed.</t>
         </is>
       </c>
-      <c r="D37" s="11" t="inlineStr">
+      <c r="D38" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="182" customHeight="1">
-      <c r="A38" s="5" t="inlineStr">
+    <row r="39" ht="182" customHeight="1">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S11(1)</t>
         </is>
       </c>
-      <c r="B38" s="11" t="inlineStr">
+      <c r="B39" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Rules, 2025, Rule 14(1) to 14(3)</t>
         </is>
       </c>
-      <c r="C38" s="11" t="inlineStr">
+      <c r="C39" s="11" t="inlineStr">
         <is>
           <t>(1) For enabling Data Principals to exercise their rights under the Act, the Data Fiduciary and, where applicable, the Consent Manager, shall prominently publish on its website or app, or both, as the case may be, — (a) the details of the means using which a Data Principal may make a request for the exercise of such rights; and (b) the particulars, if any, such as the username or other identifier of such a Data Principal, which may be required to identify her under its terms of service. (2) To exercise the rights of the Data Principal under the Act, she may make a request to the Data Fiduciary to whom she has previously given consent for processing of her personal data, using the means and furnishing the particulars required by such Data Fiduciary for the exercise of such rights. (3) Every Data Fiduciary and Consent Manager shall prominently publish on its website or app, or both, as the case may be, within a reasonable period not exceeding ninety days under its grievance redressal system for responding to the grievances of Data Principals and shall, for ensuring the effectiveness of the system in responding within such period, implement appropriate technical and organisational measures.</t>
         </is>
       </c>
-      <c r="D38" s="11" t="inlineStr">
+      <c r="D39" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="70" customHeight="1">
-      <c r="A39" s="5" t="inlineStr">
+    <row r="40" ht="70" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S11(1)</t>
         </is>
       </c>
-      <c r="B39" s="11" t="inlineStr">
+      <c r="B40" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Act, 2023, Section 11(2)</t>
         </is>
       </c>
-      <c r="C39" s="11" t="inlineStr">
+      <c r="C40" s="11" t="inlineStr">
         <is>
           <t>(2) Nothing contained in clause (b) or clause (c) of sub-section (1) shall apply in respect of the sharing of any personal data by the said Data Fiduciary with any other Data Fiduciary authorised by law to obtain such personal data, where such sharing is pursuant to a request made in writing by such other Data Fiduciary for the purpose of prevention or detection or investigation of offences or cyber incidents, or for prosecution or punishment of offences.</t>
         </is>
       </c>
-      <c r="D39" s="11" t="inlineStr">
+      <c r="D40" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="140" customHeight="1">
-      <c r="A40" s="5" t="inlineStr">
+    <row r="41" ht="140" customHeight="1">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S12</t>
         </is>
       </c>
-      <c r="B40" s="11" t="inlineStr">
+      <c r="B41" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Act, 2023, Section 12(1) to 12(3)</t>
         </is>
       </c>
-      <c r="C40" s="11" t="inlineStr">
+      <c r="C41" s="11" t="inlineStr">
         <is>
           <t>(1) A Data Principal shall have the right to correction, completion, updating and erasure of her personal data for the processing of which she has previously given consent, including consent as referred to in clause (a) of section 7, in accordance with any requirement or procedure under any law for the time being in force. (2) A Data Fiduciary shall, upon receiving a request for correction, completion or updating from a Data Principal,— (a) correct the inaccurate or misleading personal data; (b) complete the incomplete personal data; and (c) update the personal data. (3) A Data Principal shall make a request in such manner as may be prescribed to the Data Fiduciary for erasure of her personal data, and upon receipt of such a request, the Data Fiduciary shall erase her personal data unless retention of the same is necessary for the specified purpose or for compliance with any law for the time being in force.</t>
         </is>
       </c>
-      <c r="D40" s="11" t="inlineStr">
+      <c r="D41" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="182" customHeight="1">
-      <c r="A41" s="5" t="inlineStr">
+    <row r="42" ht="182" customHeight="1">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S12</t>
         </is>
       </c>
-      <c r="B41" s="11" t="inlineStr">
+      <c r="B42" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Rules, 2025, Rule 14(1) to 14(3)</t>
         </is>
       </c>
-      <c r="C41" s="11" t="inlineStr">
+      <c r="C42" s="11" t="inlineStr">
         <is>
           <t>(1) For enabling Data Principals to exercise their rights under the Act, the Data Fiduciary and, where applicable, the Consent Manager, shall prominently publish on its website or app, or both, as the case may be, — (a) the details of the means using which a Data Principal may make a request for the exercise of such rights; and (b) the particulars, if any, such as the username or other identifier of such a Data Principal, which may be required to identify her under its terms of service. (2) To exercise the rights of the Data Principal under the Act, she may make a request to the Data Fiduciary to whom she has previously given consent for processing of her personal data, using the means and furnishing the particulars required by such Data Fiduciary for the exercise of such rights. (3) Every Data Fiduciary and Consent Manager shall prominently publish on its website or app, or both, as the case may be, within a reasonable period not exceeding ninety days under its grievance redressal system for responding to the grievances of Data Principals and shall, for ensuring the effectiveness of the system in responding within such period, implement appropriate technical and organisational measures.</t>
         </is>
       </c>
-      <c r="D41" s="11" t="inlineStr">
+      <c r="D42" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="45" customHeight="1">
-      <c r="A42" s="5" t="inlineStr">
+    <row r="43" ht="45" customHeight="1">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S13</t>
         </is>
       </c>
-      <c r="B42" s="11" t="inlineStr">
+      <c r="B43" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Act, 2023, Section 8(10)</t>
         </is>
       </c>
-      <c r="C42" s="11" t="inlineStr">
+      <c r="C43" s="11" t="inlineStr">
         <is>
           <t>(10) A Data Fiduciary shall establish an effective mechanism to redress the grievances of Data Principals.</t>
         </is>
       </c>
-      <c r="D42" s="11" t="inlineStr">
+      <c r="D43" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="126" customHeight="1">
-      <c r="A43" s="5" t="inlineStr">
+    <row r="44" ht="126" customHeight="1">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S13</t>
         </is>
       </c>
-      <c r="B43" s="11" t="inlineStr">
+      <c r="B44" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Act, 2023, Section 13(1) to 13(3)</t>
         </is>
       </c>
-      <c r="C43" s="11" t="inlineStr">
+      <c r="C44" s="11" t="inlineStr">
         <is>
           <t>(1) A Data Principal shall have the right to have readily available means of grievance redressal provided by a Data Fiduciary or Consent Manager in respect of any act or omission of such Data Fiduciary or Consent Manager regarding the performance of its obligations in relation to the personal data of such Data Principal or the exercise of her rights under the provisions of this Act and the rules made thereunder. (2) The Data Fiduciary or Consent Manager shall respond to any grievances referred to in sub-section (1) within such period as may be prescribed from the date of its receipt for all or any class of Data Fiduciaries. (3) The Data Principal shall exhaust the opportunity of redressing her grievance under this section before approaching the Board.</t>
         </is>
       </c>
-      <c r="D43" s="11" t="inlineStr">
+      <c r="D44" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="182" customHeight="1">
-      <c r="A44" s="5" t="inlineStr">
+    <row r="45" ht="182" customHeight="1">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S13</t>
         </is>
       </c>
-      <c r="B44" s="11" t="inlineStr">
+      <c r="B45" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Rules, 2025, Rule 14(1) to 14(3)</t>
         </is>
       </c>
-      <c r="C44" s="11" t="inlineStr">
+      <c r="C45" s="11" t="inlineStr">
         <is>
           <t>(1) For enabling Data Principals to exercise their rights under the Act, the Data Fiduciary and, where applicable, the Consent Manager, shall prominently publish on its website or app, or both, as the case may be, — (a) the details of the means using which a Data Principal may make a request for the exercise of such rights; and (b) the particulars, if any, such as the username or other identifier of such a Data Principal, which may be required to identify her under its terms of service. (2) To exercise the rights of the Data Principal under the Act, she may make a request to the Data Fiduciary to whom she has previously given consent for processing of her personal data, using the means and furnishing the particulars required by such Data Fiduciary for the exercise of such rights. (3) Every Data Fiduciary and Consent Manager shall prominently publish on its website or app, or both, as the case may be, within a reasonable period not exceeding ninety days under its grievance redressal system for responding to the grievances of Data Principals and shall, for ensuring the effectiveness of the system in responding within such period, implement appropriate technical and organisational measures.</t>
         </is>
       </c>
-      <c r="D44" s="11" t="inlineStr">
+      <c r="D45" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="56" customHeight="1">
-      <c r="A45" s="5" t="inlineStr">
+    <row r="46" ht="56" customHeight="1">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S14(1)</t>
         </is>
       </c>
-      <c r="B45" s="11" t="inlineStr">
+      <c r="B46" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Act, 2023, Section 14(1)</t>
         </is>
       </c>
-      <c r="C45" s="11" t="inlineStr">
+      <c r="C46" s="11" t="inlineStr">
         <is>
           <t>(1) A Data Principal shall have the right to nominate, in such manner as may be prescribed, any other individual, who shall, in the event of death or incapacity of the Data Principal, exercise the rights of the Data Principal in accordance with the provisions of this Act and the rules made thereunder.</t>
         </is>
       </c>
-      <c r="D45" s="11" t="inlineStr">
+      <c r="D46" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="70" customHeight="1">
-      <c r="A46" s="5" t="inlineStr">
+    <row r="47" ht="70" customHeight="1">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S9(1)</t>
         </is>
       </c>
-      <c r="B46" s="11" t="inlineStr">
+      <c r="B47" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Act, 2023, Section 9(1)</t>
         </is>
       </c>
-      <c r="C46" s="11" t="inlineStr">
+      <c r="C47" s="11" t="inlineStr">
         <is>
           <t>(1) The Data Fiduciary shall, before processing any personal data of a child or a person with disability who has a lawful guardian obtain verifiable consent of the parent of such child or the lawful guardian, as the case may be, in such manner as may be prescribed. [Note: as originally enacted. The Digital Personal Data Protection (Removal of Difficulties) Order, 2026 is reported to insert the word “of” before “a person with disability”. Check the amended text.]</t>
         </is>
       </c>
-      <c r="D46" s="11" t="inlineStr">
+      <c r="D47" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="409" customHeight="1">
-      <c r="A47" s="5" t="inlineStr">
+    <row r="48" ht="409" customHeight="1">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S9(1)</t>
         </is>
       </c>
-      <c r="B47" s="11" t="inlineStr">
+      <c r="B48" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Rules, 2025, Rule 10(1), with the Illustration to Rule 10</t>
         </is>
       </c>
-      <c r="C47" s="11" t="inlineStr">
+      <c r="C48" s="11" t="inlineStr">
         <is>
           <t>(1) A Data Fiduciary shall adopt appropriate technical and organisational measures to ensure that verifiable consent of the parent is obtained before the processing of any personal data of a child and shall observe due diligence, for checking that the individual identifying herself as the parent is an adult who is identifiable if required in connection with compliance with any law for the time being in force in India, by reference to— (a) reliable details of identity and age of the individual available with the Data Fiduciary; or (b) details of identity and age, voluntarily provided — (i) by the individual; or (ii) through a virtual token mapped to such details, which is issued by an authorised entity. Illustration. C is a child, P is a parent, and DF is a Data Fiduciary. A user account of C is sought to be created on the online platform of DF, by processing the personal data of C. Case 1: C informs DF that she is a child and declares P as her parent. DF shall enable P to identify herself through its website, app or other appropriate means. P identifies herself as the parent and informs DF that she is a registered user on DF’s platform and has previously made available her identity and age details to DF. Before processing C’s personal data for the creation of her user account, DF shall check to confirm that it holds reliable identity and age details of P and that P is an identifiable adult. Case 2: C informs DF that she is a child and declares P as her parent. DF shall enable P to identify herself through its website, app or other appropriate means. P identifies herself as the parent and informs DF that she herself is not a registered user on DF’s platform. Before processing C’s personal data for the creation of her user account, DF shall, by reference to identity and age details issued by an entity entrusted by law or the Government with maintenance of the said details or to a virtual token mapped to the identity and age, check that P is an identifiable adult. P may voluntarily make such details available using the services of a Digital Locker service provider. Case 3: P is opening an account for C and identifies herself as C’s parent and informs DF that she is a registered user on DF’s platform and has previously made available her identity and age details to DF. Before processing C’s personal data for the creation of her user account, DF shall check to confirm that it holds reliable identity and age details of P and that P is an identifiable adult. Case 4: P is opening an account for C and identifies herself as C’s parent and informs DF that she herself is not a registered user on DF’s platform. Before processing C’s personal data for the creation of her user account, DF shall, by reference to identity and age details issued by an entity entrusted by law or the Government with maintenance of the said details or to a virtual token mapped to the identity and age, check that P is an identifiable adult. P may voluntarily make such details available using the services of a Digital Locker service provider.</t>
         </is>
       </c>
-      <c r="D47" s="11" t="inlineStr">
+      <c r="D48" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="45" customHeight="1">
-      <c r="A48" s="5" t="inlineStr">
+    <row r="49" ht="45" customHeight="1">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S9(3)</t>
         </is>
       </c>
-      <c r="B48" s="11" t="inlineStr">
+      <c r="B49" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Act, 2023, Section 9(2) and Section 9(3)</t>
         </is>
       </c>
-      <c r="C48" s="11" t="inlineStr">
+      <c r="C49" s="11" t="inlineStr">
         <is>
           <t>(2) A Data Fiduciary shall not undertake such processing of personal data that is likely to cause any detrimental effect on the well-being of a child. (3) A Data Fiduciary shall not undertake tracking or behavioural monitoring of children or targeted advertising directed at children.</t>
         </is>
       </c>
-      <c r="D48" s="11" t="inlineStr">
+      <c r="D49" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="98" customHeight="1">
-      <c r="A49" s="5" t="inlineStr">
+    <row r="50" ht="98" customHeight="1">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S9(3)</t>
         </is>
       </c>
-      <c r="B49" s="11" t="inlineStr">
+      <c r="B50" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Rules, 2025, Rule 12</t>
         </is>
       </c>
-      <c r="C49" s="11" t="inlineStr">
+      <c r="C50" s="11" t="inlineStr">
         <is>
           <t>12. Exemptions from certain obligations applicable to processing of personal data of child. — (1) The provisions of sub-sections (1) and (3) of section 9 of the Act shall not be applicable to processing of personal data of a child by such class of Data Fiduciaries as are specified in Part A of Fourth Schedule, subject to such conditions as are specified in the said Part. (2) The provisions of sub-sections (1) and (3) of section 9 of the Act shall not be applicable to processing of personal data of a child for such purposes as are specified in Part B of Fourth Schedule, subject to such conditions as are specified in the said Part.</t>
         </is>
       </c>
-      <c r="D49" s="11" t="inlineStr">
+      <c r="D50" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="56" customHeight="1">
-      <c r="A50" s="5" t="inlineStr">
+    <row r="51" ht="56" customHeight="1">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>DPDP-Rule-11(1)</t>
         </is>
       </c>
-      <c r="B50" s="11" t="inlineStr">
+      <c r="B51" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Rules, 2025, Rule 11(1)</t>
         </is>
       </c>
-      <c r="C50" s="11" t="inlineStr">
+      <c r="C51" s="11" t="inlineStr">
         <is>
           <t>(1) A Data Fiduciary, while obtaining verifiable consent from an individual identifying herself as the lawful guardian of a person with disability, shall observe due diligence to verify that such guardian is appointed by a court of law, or by a designated authority or by a local level committee, under the law applicable to guardianship.</t>
         </is>
       </c>
-      <c r="D50" s="11" t="inlineStr">
+      <c r="D51" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="196" customHeight="1">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>DPDP-Act-S10(2)</t>
-        </is>
-      </c>
-      <c r="B51" s="11" t="inlineStr">
-        <is>
-          <t>Digital Personal Data Protection Act, 2023, Section 10(2)</t>
-        </is>
-      </c>
-      <c r="C51" s="11" t="inlineStr">
-        <is>
-          <t>(2) The Significant Data Fiduciary shall— (a) appoint a Data Protection Officer who shall— (i) represent the Significant Data Fiduciary under the provisions of this Act; (ii) be based in India; (iii) be an individual responsible to the Board of Directors or similar governing body of the Significant Data Fiduciary; and (iv) be the point of contact for the grievance redressal mechanism under the provisions of this Act; (b) appoint an independent data auditor to carry out data audit, who shall evaluate the compliance of the Significant Data Fiduciary in accordance with the provisions of this Act; and (c) undertake the following other measures, namely:— (i) periodic Data Protection Impact Assessment, which shall be a process comprising a description of the rights of Data Principals and the purpose of processing of their personal data, assessment and management of the risk to the rights of the Data Principals, and such other matters regarding such process as may be prescribed; (ii) periodic audit; and (iii) such other measures, consistent with the provisions of this Act, as may be prescribed. [Note: as originally enacted. The Removal of Difficulties Order, 2026 is reported to replace “audit” with “data audit” in clause (c)(ii). Check the amended text.]</t>
-        </is>
-      </c>
-      <c r="D51" s="11" t="inlineStr">
-        <is>
-          <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
         </is>
       </c>
     </row>
     <row r="52" ht="196" customHeight="1">
       <c r="A52" s="5" t="inlineStr">
         <is>
+          <t>DPDP-Act-S10(2)</t>
+        </is>
+      </c>
+      <c r="B52" s="11" t="inlineStr">
+        <is>
+          <t>Digital Personal Data Protection Act, 2023, Section 10(2)</t>
+        </is>
+      </c>
+      <c r="C52" s="11" t="inlineStr">
+        <is>
+          <t>(2) The Significant Data Fiduciary shall— (a) appoint a Data Protection Officer who shall— (i) represent the Significant Data Fiduciary under the provisions of this Act; (ii) be based in India; (iii) be an individual responsible to the Board of Directors or similar governing body of the Significant Data Fiduciary; and (iv) be the point of contact for the grievance redressal mechanism under the provisions of this Act; (b) appoint an independent data auditor to carry out data audit, who shall evaluate the compliance of the Significant Data Fiduciary in accordance with the provisions of this Act; and (c) undertake the following other measures, namely:— (i) periodic Data Protection Impact Assessment, which shall be a process comprising a description of the rights of Data Principals and the purpose of processing of their personal data, assessment and management of the risk to the rights of the Data Principals, and such other matters regarding such process as may be prescribed; (ii) periodic audit; and (iii) such other measures, consistent with the provisions of this Act, as may be prescribed. [Note: as originally enacted. The Removal of Difficulties Order, 2026 is reported to replace “audit” with “data audit” in clause (c)(ii). Check the amended text.]</t>
+        </is>
+      </c>
+      <c r="D52" s="11" t="inlineStr">
+        <is>
+          <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="196" customHeight="1">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
           <t>DPDP-Rule-13</t>
         </is>
       </c>
-      <c r="B52" s="11" t="inlineStr">
+      <c r="B53" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Rules, 2025, Rule 13(1) to 13(4)</t>
         </is>
       </c>
-      <c r="C52" s="11" t="inlineStr">
+      <c r="C53" s="11" t="inlineStr">
         <is>
           <t>(1) A Significant Data Fiduciary shall, once in every period of twelve months from the date on which it is notified as such or is included in the class of Data Fiduciaries notified as such, undertake a Data Protection Impact Assessment and an audit to ensure effective observance of the provisions of this Act and the rules made thereunder. (2) A Significant Data Fiduciary shall cause the person carrying out the Data Protection Impact Assessment and audit to furnish to the Board a report containing significant observations in the Data Protection Impact Assessment and audit. (3) A Significant Data Fiduciary shall observe due diligence to verify that technical measures including algorithmic software adopted by it for hosting, display, uploading, modification, publishing, transmission, storage, updating or sharing of personal data processed by it are not likely to pose a risk to the rights of Data Principals. (4) A Significant Data Fiduciary shall undertake measures to ensure that personal data specified by the Central Government, on the basis of the recommendations of a committee constituted by it, is processed subject to the restriction that the personal data and the traffic data pertaining to its flow is not transferred outside the territory of India.</t>
         </is>
       </c>
-      <c r="D52" s="11" t="inlineStr">
+      <c r="D53" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="84" customHeight="1">
-      <c r="A53" s="5" t="inlineStr">
+    <row r="54" ht="84" customHeight="1">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S16</t>
         </is>
       </c>
-      <c r="B53" s="11" t="inlineStr">
+      <c r="B54" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Act, 2023, Section 16(1) and Section 16(2)</t>
         </is>
       </c>
-      <c r="C53" s="11" t="inlineStr">
+      <c r="C54" s="11" t="inlineStr">
         <is>
           <t>(1) The Central Government may, by notification, restrict the transfer of personal data by a Data Fiduciary for processing to such country or territory outside India as may be so notified. (2) Nothing contained in this section shall restrict the applicability of any law for the time being in force in India that provides for a higher degree of protection for or restriction on transfer of personal data by a Data Fiduciary outside India in relation to any personal data or Data Fiduciary or class thereof.</t>
         </is>
       </c>
-      <c r="D53" s="11" t="inlineStr">
+      <c r="D54" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="70" customHeight="1">
-      <c r="A54" s="5" t="inlineStr">
+    <row r="55" ht="70" customHeight="1">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S16</t>
         </is>
       </c>
-      <c r="B54" s="11" t="inlineStr">
+      <c r="B55" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Rules, 2025, Rule 15</t>
         </is>
       </c>
-      <c r="C54" s="11" t="inlineStr">
+      <c r="C55" s="11" t="inlineStr">
         <is>
           <t>15. Transfer of personal data outside the territory of India.— Any personal data processed by a Data Fiduciary under the Act may be transferred outside the territory of India subject to the restriction that the Data Fiduciary shall meet such requirements as the Central Government may, by general or special order, specify in respect of making such personal data available to any foreign State, or to any person or entity under the control of or any agency of such a State.</t>
         </is>
       </c>
-      <c r="D54" s="11" t="inlineStr">
+      <c r="D55" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="45" customHeight="1">
-      <c r="A55" s="5" t="inlineStr">
+    <row r="56" ht="45" customHeight="1">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>DPDP-Rule-23</t>
         </is>
       </c>
-      <c r="B55" s="11" t="inlineStr">
+      <c r="B56" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Act, 2023, Section 36</t>
         </is>
       </c>
-      <c r="C55" s="11" t="inlineStr">
+      <c r="C56" s="11" t="inlineStr">
         <is>
           <t>The Central Government may, for the purposes of this Act, require the Board and any Data Fiduciary or intermediary to furnish such information as it may call for.</t>
         </is>
       </c>
-      <c r="D55" s="11" t="inlineStr">
+      <c r="D56" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="112" customHeight="1">
-      <c r="A56" s="5" t="inlineStr">
-        <is>
-          <t>DPDP-Rule-23</t>
-        </is>
-      </c>
-      <c r="B56" s="11" t="inlineStr">
-        <is>
-          <t>Digital Personal Data Protection Rules, 2025, Rule 23(1) and 23(2)</t>
-        </is>
-      </c>
-      <c r="C56" s="11" t="inlineStr">
-        <is>
-          <t>(1) The Central Government may, for such purposes of the Act as are specified in Seventh Schedule, acting through the corresponding authorised person specified in the said Schedule, require any Data Fiduciary or intermediary to furnish such information as may be called for, within the specified period as may be given in such. (2) Where the disclosure of furnishing of information as referred to in sub-rule (1) is likely to prejudicially affect the sovereignty and integrity of India or security of the State, the Central Government may require the Data Fiduciary or intermediary to not disclose such furnishing to affected Data Principal or any other person except with the previous permission, in writing, of the authorised person.</t>
-        </is>
-      </c>
-      <c r="D56" s="11" t="inlineStr">
-        <is>
-          <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
         </is>
       </c>
     </row>
     <row r="57" ht="112" customHeight="1">
       <c r="A57" s="5" t="inlineStr">
         <is>
+          <t>DPDP-Rule-23</t>
+        </is>
+      </c>
+      <c r="B57" s="11" t="inlineStr">
+        <is>
+          <t>Digital Personal Data Protection Rules, 2025, Rule 23(1) and 23(2)</t>
+        </is>
+      </c>
+      <c r="C57" s="11" t="inlineStr">
+        <is>
+          <t>(1) The Central Government may, for such purposes of the Act as are specified in Seventh Schedule, acting through the corresponding authorised person specified in the said Schedule, require any Data Fiduciary or intermediary to furnish such information as may be called for, within the specified period as may be given in such. (2) Where the disclosure of furnishing of information as referred to in sub-rule (1) is likely to prejudicially affect the sovereignty and integrity of India or security of the State, the Central Government may require the Data Fiduciary or intermediary to not disclose such furnishing to affected Data Principal or any other person except with the previous permission, in writing, of the authorised person.</t>
+        </is>
+      </c>
+      <c r="D57" s="11" t="inlineStr">
+        <is>
+          <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="56" customHeight="1">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
           <t>DPDP-Act-S32</t>
         </is>
       </c>
-      <c r="B57" s="11" t="inlineStr">
+      <c r="B58" s="11" t="inlineStr">
+        <is>
+          <t>Digital Personal Data Protection Act, 2023, Section 27(2)</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="inlineStr">
+        <is>
+          <t>(2) The Board may, for the effective discharge of its functions under the provisions of this Act, after giving the person concerned an opportunity of being heard and after recording reasons in writing, issue such directions as it may consider necessary to such person, who shall be bound to comply with the same.</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="112" customHeight="1">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>DPDP-Act-S32</t>
+        </is>
+      </c>
+      <c r="B59" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Act, 2023, Section 32(1), 32(4) and 32(5)</t>
         </is>
       </c>
-      <c r="C57" s="11" t="inlineStr">
+      <c r="C59" s="11" t="inlineStr">
         <is>
           <t>(1) The Board may accept a voluntary undertaking in respect of any matter related to observance of the provisions of this Act from any person at any stage of a proceeding under section 28. … (4) The acceptance of the voluntary undertaking by the Board shall constitute a bar on proceedings under the provisions of this Act as regards the contents of the voluntary undertaking, except in cases covered by sub-section (5). (5) Where a person fails to adhere to any term of the voluntary undertaking accepted by the Board, such breach shall be deemed to be breach of the provisions of this Act and the Board may, after giving such person an opportunity of being heard, proceed in accordance with the provisions of section 33.</t>
         </is>
       </c>
-      <c r="D57" s="11" t="inlineStr">
+      <c r="D59" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="45" customHeight="1">
-      <c r="A58" s="5" t="inlineStr">
+    <row r="60" ht="45" customHeight="1">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S32</t>
         </is>
       </c>
-      <c r="B58" s="11" t="inlineStr">
+      <c r="B60" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Act, 2023, Section 29(2)</t>
         </is>
       </c>
-      <c r="C58" s="11" t="inlineStr">
+      <c r="C60" s="11" t="inlineStr">
         <is>
           <t>(2) Every appeal under sub-section (1) shall be filed within a period of sixty days from the date of receipt of the order or direction appealed against and it shall be in such form and manner and shall be accompanied by such fee as may be prescribed.</t>
         </is>
       </c>
-      <c r="D58" s="11" t="inlineStr">
+      <c r="D60" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="45" customHeight="1">
-      <c r="A59" s="5" t="inlineStr">
+    <row r="61" ht="45" customHeight="1">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S32</t>
         </is>
       </c>
-      <c r="B59" s="11" t="inlineStr">
+      <c r="B61" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Rules, 2025, Rule 22(1)</t>
         </is>
       </c>
-      <c r="C59" s="11" t="inlineStr">
+      <c r="C61" s="11" t="inlineStr">
         <is>
           <t>(1) Any person aggrieved by an order or direction of the Board, may prefer an appeal before the Appellate Tribunal, it shall be filed in digital form as the Appellate Tribunal may decide.</t>
         </is>
       </c>
-      <c r="D59" s="11" t="inlineStr">
+      <c r="D61" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="56" customHeight="1">
-      <c r="A60" s="5" t="inlineStr">
+    <row r="62" ht="56" customHeight="1">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S17(2)(b)</t>
         </is>
       </c>
-      <c r="B60" s="11" t="inlineStr">
+      <c r="B62" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Act, 2023, Section 17(2)(b)</t>
         </is>
       </c>
-      <c r="C60" s="11" t="inlineStr">
+      <c r="C62" s="11" t="inlineStr">
         <is>
           <t>(2) The provisions of this Act shall not apply in respect of the processing of personal data— … (b) necessary for research, archiving or statistical purposes if the personal data is not to be used to take any decision specific to a Data Principal and such processing is carried on in accordance with such standards as may be prescribed.</t>
         </is>
       </c>
-      <c r="D60" s="11" t="inlineStr">
+      <c r="D62" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="56" customHeight="1">
-      <c r="A61" s="5" t="inlineStr">
+    <row r="63" ht="56" customHeight="1">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S17(2)(b)</t>
         </is>
       </c>
-      <c r="B61" s="11" t="inlineStr">
+      <c r="B63" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Rules, 2025, Rule 16</t>
         </is>
       </c>
-      <c r="C61" s="11" t="inlineStr">
+      <c r="C63" s="11" t="inlineStr">
         <is>
           <t>16. Exemption from Act for research, archiving or statistical purposes. —The provisions of the Act shall not apply to the processing of personal data necessary for research, archiving or statistical purposes if it is carried on in accordance with the standards specified in Second Schedule.</t>
         </is>
       </c>
-      <c r="D61" s="11" t="inlineStr">
+      <c r="D63" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 3(i), G.S.R. 846(E), 13 November 2025</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="294" customHeight="1">
-      <c r="A62" s="5" t="inlineStr">
+    <row r="64" ht="294" customHeight="1">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S17(1)</t>
         </is>
       </c>
-      <c r="B62" s="11" t="inlineStr">
+      <c r="B64" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Act, 2023, Section 17(1)</t>
         </is>
       </c>
-      <c r="C62" s="11" t="inlineStr">
+      <c r="C64" s="11" t="inlineStr">
         <is>
           <t>17. (1) The provisions of Chapter II, except sub-sections (1) and (5) of section 8, and those of Chapter III and section 16 shall not apply where— (a) the processing of personal data is necessary for enforcing any legal right or claim; (b) the processing of personal data by any court or tribunal or any other body in India which is entrusted by law with the performance of any judicial or quasi-judicial or regulatory or supervisory function, where such processing is necessary for the performance of such function; (c) personal data is processed in the interest of prevention, detection, investigation or prosecution of any offence or contravention of any law for the time being in force in India; (d) personal data of Data Principals not within the territory of India is processed pursuant to any contract entered into with any person outside the territory of India by any person based in India; (e) the processing is necessary for a scheme of compromise or arrangement or merger or amalgamation of two or more companies or a reconstruction by way of demerger or otherwise of a company, or transfer of undertaking of one or more company to another company, or involving division of one or more companies, approved by a court or tribunal or other authority competent to do so by any law for the time being in force; and (f) the processing is for the purpose of ascertaining the financial information and assets and liabilities of any person who has defaulted in payment due on account of a loan or advance taken from a financial institution, subject to such processing being in accordance with the provisions regarding disclosure of information or data in any other law for the time being in force. Explanation.—For the purposes of this clause, the expressions "default" and "financial institution" shall have the meanings respectively assigned to them in sub-sections (12) and (14) of section 3 of the Insolvency and Bankruptcy Code, 2016.</t>
         </is>
       </c>
-      <c r="D62" s="11" t="inlineStr">
+      <c r="D64" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="98" customHeight="1">
-      <c r="A63" s="5" t="inlineStr">
+    <row r="65" ht="98" customHeight="1">
+      <c r="A65" s="5" t="inlineStr">
         <is>
           <t>DPDP-Act-S17(1)</t>
         </is>
       </c>
-      <c r="B63" s="11" t="inlineStr">
+      <c r="B65" s="11" t="inlineStr">
         <is>
           <t>Digital Personal Data Protection Act, 2023, Section 17(3) and Section 17(5)</t>
         </is>
       </c>
-      <c r="C63" s="11" t="inlineStr">
+      <c r="C65" s="11" t="inlineStr">
         <is>
           <t>(3) The Central Government may, having regard to the volume and nature of personal data processed, notify certain Data Fiduciaries or class of Data Fiduciaries, including startups, as Data Fiduciaries to whom the provisions of section 5, sub-sections (3) and (7) of section 8 and sections 10 and 11 shall not apply. … (5) The Central Government may, before expiry of five years from the date of commencement of this Act, by notification, declare that any provision of this Act shall not apply to such Data Fiduciary or classes of Data Fiduciaries for such period as may be specified in the notification.</t>
         </is>
       </c>
-      <c r="D63" s="11" t="inlineStr">
+      <c r="D65" s="11" t="inlineStr">
         <is>
           <t>Gazette of India, Extraordinary, Part II, Section 1, No. 25, 11 August 2023</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:D63"/>
+  <autoFilter ref="A4:D65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader/>
@@ -9136,7 +9180,7 @@
       </c>
       <c r="G16" s="36" t="inlineStr">
         <is>
-          <t>Binds Consent Managers; a company must accept consent actions made through them.</t>
+          <t>Gives the person the right to give, manage, review or withdraw consent through a Consent Manager; binds Consent Managers.</t>
         </is>
       </c>
     </row>
@@ -9229,7 +9273,7 @@
       </c>
       <c r="E19" s="30" t="inlineStr">
         <is>
-          <t>Grouped in DPDP-Act-S7</t>
+          <t>Not included (the State only)</t>
         </is>
       </c>
       <c r="F19" s="30" t="inlineStr">
@@ -9246,12 +9290,12 @@
     <row r="20" ht="40" customHeight="1">
       <c r="A20" s="33" t="inlineStr">
         <is>
-          <t>Act s.8(1), 8(2)</t>
+          <t>Act s.8(1), 8(2), 8(4)</t>
         </is>
       </c>
       <c r="B20" s="34" t="inlineStr">
         <is>
-          <t>Accountability; processors only under a valid contract</t>
+          <t>Accountability; processors only under a valid contract; measures to ensure the Act is observed</t>
         </is>
       </c>
       <c r="C20" s="34" t="inlineStr">
@@ -9312,12 +9356,12 @@
     <row r="22" ht="40" customHeight="1">
       <c r="A22" s="33" t="inlineStr">
         <is>
-          <t>Act s.8(4), 8(5)</t>
+          <t>Act s.8(5)</t>
         </is>
       </c>
       <c r="B22" s="34" t="inlineStr">
         <is>
-          <t>Technical and organisational measures; security safeguards</t>
+          <t>Security safeguards</t>
         </is>
       </c>
       <c r="C22" s="34" t="inlineStr">
@@ -9940,7 +9984,7 @@
       </c>
       <c r="G40" s="30" t="inlineStr">
         <is>
-          <t>Binds individuals, not companies (penalty up to ₹10,000). Recommended: Coverage note only, no row (sheet 3).</t>
+          <t>Binds individuals, not companies (penalty up to ₹10,000).</t>
         </is>
       </c>
     </row>
@@ -10245,12 +10289,12 @@
       </c>
       <c r="C49" s="36" t="inlineStr">
         <is>
-          <t>Board</t>
+          <t>Board; any person it directs</t>
         </is>
       </c>
       <c r="D49" s="36" t="inlineStr">
         <is>
-          <t>Indirectly</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E49" s="36" t="inlineStr">
@@ -10265,7 +10309,7 @@
       </c>
       <c r="G49" s="36" t="inlineStr">
         <is>
-          <t>A company is subject to these powers; listed for reference.</t>
+          <t>A person given a direction by the Board is bound to comply with it (s.27(2)).</t>
         </is>
       </c>
     </row>
@@ -10406,37 +10450,37 @@
       <c r="G53" s="34" t="inlineStr"/>
     </row>
     <row r="54" ht="40" customHeight="1">
-      <c r="A54" s="22" t="inlineStr">
+      <c r="A54" s="35" t="inlineStr">
         <is>
           <t>Act s.33 and the Schedule</t>
         </is>
       </c>
-      <c r="B54" s="30" t="inlineStr">
+      <c r="B54" s="36" t="inlineStr">
         <is>
           <t>Penalties</t>
         </is>
       </c>
-      <c r="C54" s="30" t="inlineStr">
+      <c r="C54" s="36" t="inlineStr">
         <is>
           <t>Any person in breach</t>
         </is>
       </c>
-      <c r="D54" s="30" t="inlineStr">
+      <c r="D54" s="36" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E54" s="30" t="inlineStr">
-        <is>
-          <t>Penalties sheet; grouped in DPDP-Act-S32</t>
-        </is>
-      </c>
-      <c r="F54" s="30" t="inlineStr">
-        <is>
-          <t>Does not apply to companies</t>
-        </is>
-      </c>
-      <c r="G54" s="30" t="inlineStr"/>
+      <c r="E54" s="36" t="inlineStr">
+        <is>
+          <t>Grouped in DPDP-Act-S32; amounts on the Penalties sheet</t>
+        </is>
+      </c>
+      <c r="F54" s="36" t="inlineStr">
+        <is>
+          <t>Grouped in a row</t>
+        </is>
+      </c>
+      <c r="G54" s="36" t="inlineStr"/>
     </row>
     <row r="55" ht="40" customHeight="1">
       <c r="A55" s="22" t="inlineStr">
@@ -10541,7 +10585,7 @@
       </c>
       <c r="G57" s="30" t="inlineStr">
         <is>
-          <t>Applies where the company is an intermediary, after a Board reference. Noted for intermediaries; no row recommended.</t>
+          <t>Applies only where the company is an intermediary, after a reference by the Board.</t>
         </is>
       </c>
     </row>
@@ -10738,7 +10782,7 @@
       </c>
       <c r="B63" s="34" t="inlineStr">
         <is>
-          <t>Amendment of the IT Act: Section 43A and Section 87(2)(ob) omitted</t>
+          <t>Amendment of the IT Act: Section 43A omitted; the DPDP Act added to the proviso to Section 81; Section 87(2)(ob) omitted</t>
         </is>
       </c>
       <c r="C63" s="34" t="inlineStr">
@@ -11292,7 +11336,7 @@
     <row r="80" ht="40" customHeight="1">
       <c r="A80" s="35" t="inlineStr">
         <is>
-          <t>Rule 12(1) to 12(3); Fourth Schedule</t>
+          <t>Rule 12(1), 12(2); Fourth Schedule</t>
         </is>
       </c>
       <c r="B80" s="36" t="inlineStr">
@@ -11312,7 +11356,7 @@
       </c>
       <c r="E80" s="36" t="inlineStr">
         <is>
-          <t>Grouped in DPDP-Act-S9(3)</t>
+          <t>Grouped in DPDP-Act-S9(3); also lifts s.9(1)</t>
         </is>
       </c>
       <c r="F80" s="36" t="inlineStr">
@@ -11368,7 +11412,7 @@
       </c>
       <c r="C82" s="36" t="inlineStr">
         <is>
-          <t>Data Fiduciary</t>
+          <t>Data Fiduciary; Consent Manager (Rule 14(1))</t>
         </is>
       </c>
       <c r="D82" s="36" t="inlineStr">
@@ -11401,7 +11445,7 @@
       </c>
       <c r="C83" s="36" t="inlineStr">
         <is>
-          <t>Data Fiduciary</t>
+          <t>Data Fiduciary; Consent Manager</t>
         </is>
       </c>
       <c r="D83" s="36" t="inlineStr">
@@ -11663,7 +11707,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Version 2 replaced the working codes of version 1 with identifiers from the law's own numbering. Version 3 (14 October 2026, revised 15 October 2026) adds ten rows and the column 'Provisions covered in this row'.</t>
+          <t>Version 2 replaced the working codes of version 1 with identifiers from the law's own numbering. Version 3 (14 October 2026, revised 15 October 2026, v0.1.3) adds ten rows and the column 'Provisions covered in this row'.</t>
         </is>
       </c>
     </row>
@@ -11729,7 +11773,7 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Version 2: identifier follows the numbering of the Act or the Rules so that it can be checked against the Gazette.</t>
+          <t>Version 2: identifier follows the numbering of the Act or the Rules so that it can be checked against the Gazette. v0.1.3: s.7(b) and s.7(c) removed from 'Provisions covered'; they bind only the State.</t>
         </is>
       </c>
     </row>
@@ -11751,7 +11795,7 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>Version 2: identifier follows the numbering of the Act or the Rules so that it can be checked against the Gazette.</t>
+          <t>Version 2: identifier follows the numbering of the Act or the Rules so that it can be checked against the Gazette. v0.1.3: s.6(3) contact details and the language option of s.5(3) stated in full.</t>
         </is>
       </c>
     </row>
@@ -11773,7 +11817,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Version 2: identifier follows the numbering of the Act or the Rules so that it can be checked against the Gazette.</t>
+          <t>Version 2: identifier follows the numbering of the Act or the Rules so that it can be checked against the Gazette. v0.1.3: cross-reference to Rule 3 added.</t>
         </is>
       </c>
     </row>
@@ -11883,7 +11927,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>Version 3: Rule 6(1)(f) now has its own row and is shown as a cross-reference here.</t>
+          <t>Version 3: Rule 6(1)(f) now has its own row and is shown as a cross-reference here. v0.1.3: s.8(4) (measures to ensure the whole Act is observed) moved here from DPDP-Act-S8(5).</t>
         </is>
       </c>
     </row>
@@ -11971,7 +12015,7 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Version 3: now the overall duty; each Rule 6(1) clause has its own row.</t>
+          <t>Version 3: now the overall duty; each Rule 6(1) clause has its own row. v0.1.3: s.8(4) moved to DPDP-Act-S8(1); this row now covers the security duty in s.8(5) only.</t>
         </is>
       </c>
     </row>
@@ -12301,7 +12345,7 @@
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Version 3 correction: main provision now reads Section 12(1) to 12(3); s.12(2) (duty to correct, complete and update) added to the legal text.</t>
+          <t>Version 3 correction: main provision now reads Section 12(1) to 12(3); s.12(2) (duty to correct, complete and update) added to the legal text. v0.1.3: Rules 14(1) and 14(2) added to 'Provisions covered'.</t>
         </is>
       </c>
     </row>
@@ -12367,7 +12411,7 @@
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>Version 3 (15 October 2026): the Illustration printed under Rule 10 in the Gazette added to the legal text.</t>
+          <t>Version 3 (15 October 2026): the Illustration printed under Rule 10 in the Gazette added to the legal text. v0.1.3: persons with disability who have a lawful guardian named in the requirement.</t>
         </is>
       </c>
     </row>
@@ -12389,7 +12433,7 @@
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Version 2: identifier follows the numbering of the Act or the Rules so that it can be checked against the Gazette.</t>
+          <t>Version 2: identifier follows the numbering of the Act or the Rules so that it can be checked against the Gazette. v0.1.3: Rule 12 citation corrected to 12(1), 12(2); wording makes clear that no exemption lifts the s.9(2) duty.</t>
         </is>
       </c>
     </row>
@@ -12521,7 +12565,7 @@
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Version 2: identifier follows the numbering of the Act or the Rules so that it can be checked against the Gazette.</t>
+          <t>Version 2: identifier follows the numbering of the Act or the Rules so that it can be checked against the Gazette. v0.1.3: duty to comply with Board directions (s.27(2)) added to the requirement and the legal text.</t>
         </is>
       </c>
     </row>

</xml_diff>